<commit_message>
Update example test file UsingPhonetics
Update reference test file for example UsingPhonetics. After style
infrastructure switch, the styles part is saved differently.

In addition, the original file had default formatting set to Calibri 8
(=same font as phonetics). That is wrong, because it the example
doesn't change default formatting set to Calibri 11. The default
formating font affects various things, including size of each cell.
Because old test file used only 8 points, the cells were smaller that
they should be.

After new styles part, the cells are now correct size
while ponetics remain the expected Calibri 8.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Styles/UsingPhonetics.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Styles/UsingPhonetics.xlsx
@@ -32,74 +32,64 @@
     <x:rPh sb="8" eb="9">
       <x:t>き</x:t>
     </x:rPh>
-    <x:phoneticPr fontId="0"/>
+    <x:phoneticPr fontId="1"/>
   </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="2">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="8"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>